<commit_message>
Změny 30. 3. 2026 (téměř finální)
Nahrávání článku z .txt souboru
Úprava práv:
- Editor může mazat pouze svoje články
- Moderátor může mazat články editora, ale ne admina
- V editor_app:
    - Editor může pracovat pouze se svými články, admin může upravovat všechny
    - Ve statistikách je nově počet unikátních zobrazení (podle uživatele)
</commit_message>
<xml_diff>
--- a/Uziv_Prava.xlsx
+++ b/Uziv_Prava.xlsx
@@ -247,9 +247,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -264,7 +263,7 @@
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="2">
     <dxf>
       <font>
         <b/>
@@ -286,67 +285,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <u val="none"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <u val="none"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <u val="none"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -689,164 +627,164 @@
   <sheetData>
     <row r="2" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="10" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F7" s="2" t="s">
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="C11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C4:F11">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Y">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Y">
       <formula>NOT(ISERROR(SEARCH("Y",C4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",C4)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>